<commit_message>
fix sushi erreur 2c363353389020f381a20465aebf3dc955873136
</commit_message>
<xml_diff>
--- a/SBM-corps-FHIR/ig/StructureDefinition-fr-acte-biologie-prescrit.xlsx
+++ b/SBM-corps-FHIR/ig/StructureDefinition-fr-acte-biologie-prescrit.xlsx
@@ -45,7 +45,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Observation - Fr Observation Acte biologie prescrit</t>
+    <t>Observation - Fr Acte biologie prescrit</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-08-25T15:49:50+00:00</t>
+    <t>2025-09-03T12:41:15+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -562,7 +562,7 @@
     <t>required</t>
   </si>
   <si>
-    <t>http://terminology.hl7.org/ValueSet/v3-ActPriority</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-hl7-v3-ActPriority-cisis</t>
   </si>
   <si>
     <t>Extension.value[x]</t>
@@ -1418,7 +1418,7 @@
 </t>
   </si>
   <si>
-    <t>Specimen used for this observation</t>
+    <t>Prélèvement</t>
   </si>
   <si>
     <t>The specimen that was used when this observation was made.</t>
@@ -2206,7 +2206,7 @@
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="54.6171875" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="43.21484375" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="53.1953125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>

</xml_diff>

<commit_message>
MAJ des profils FHIR 5f1c9487972ddf3be5bd28ae1930cfe9fa141f9c
</commit_message>
<xml_diff>
--- a/SBM-corps-FHIR/ig/StructureDefinition-fr-acte-biologie-prescrit.xlsx
+++ b/SBM-corps-FHIR/ig/StructureDefinition-fr-acte-biologie-prescrit.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-09-03T12:41:15+00:00</t>
+    <t>2025-09-04T10:23:02+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -481,7 +481,7 @@
     <t>Urgence</t>
   </si>
   <si>
-    <t>Indique la priorité clinique de l’observation.</t>
+    <t>Extension permettant d’indiquer d'indique la priorité clinique de l’observation.</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1

</xml_diff>